<commit_message>
Last Analysis + Writing
</commit_message>
<xml_diff>
--- a/Material/2. Interviews & Surveys/3. Quantitative Survey/attributes_for_clustering.xlsx
+++ b/Material/2. Interviews & Surveys/3. Quantitative Survey/attributes_for_clustering.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K123"/>
+  <dimension ref="A1:K126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4750,6 +4750,111 @@
         <v>8</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B124" t="n">
+        <v>7</v>
+      </c>
+      <c r="C124" t="n">
+        <v>6</v>
+      </c>
+      <c r="D124" t="n">
+        <v>10</v>
+      </c>
+      <c r="E124" t="n">
+        <v>2</v>
+      </c>
+      <c r="F124" t="n">
+        <v>1</v>
+      </c>
+      <c r="G124" t="n">
+        <v>9</v>
+      </c>
+      <c r="H124" t="n">
+        <v>3</v>
+      </c>
+      <c r="I124" t="n">
+        <v>8</v>
+      </c>
+      <c r="J124" t="n">
+        <v>4</v>
+      </c>
+      <c r="K124" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>123</v>
+      </c>
+      <c r="B125" t="n">
+        <v>8</v>
+      </c>
+      <c r="C125" t="n">
+        <v>2</v>
+      </c>
+      <c r="D125" t="n">
+        <v>6</v>
+      </c>
+      <c r="E125" t="n">
+        <v>9</v>
+      </c>
+      <c r="F125" t="n">
+        <v>7</v>
+      </c>
+      <c r="G125" t="n">
+        <v>4</v>
+      </c>
+      <c r="H125" t="n">
+        <v>5</v>
+      </c>
+      <c r="I125" t="n">
+        <v>3</v>
+      </c>
+      <c r="J125" t="n">
+        <v>1</v>
+      </c>
+      <c r="K125" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B126" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" t="n">
+        <v>10</v>
+      </c>
+      <c r="D126" t="n">
+        <v>5</v>
+      </c>
+      <c r="E126" t="n">
+        <v>6</v>
+      </c>
+      <c r="F126" t="n">
+        <v>7</v>
+      </c>
+      <c r="G126" t="n">
+        <v>2</v>
+      </c>
+      <c r="H126" t="n">
+        <v>8</v>
+      </c>
+      <c r="I126" t="n">
+        <v>1</v>
+      </c>
+      <c r="J126" t="n">
+        <v>4</v>
+      </c>
+      <c r="K126" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>